<commit_message>
Unifica la lista del Dr. Sergio Durán con la dotación básica
Agrega papelería, aseo, botiquín, caja menor y kit de retiro de puntos con valores aproximados; marca como 'Ambas' los ítems repetidos y añade multiplicador de consultorios en el Resumen. Incluye el script que genera el Excel.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012arGo69LQWzCgCo2qvwsQB
</commit_message>
<xml_diff>
--- a/cotizaciones/dotacion_consultorio_medicina_general.xlsx
+++ b/cotizaciones/dotacion_consultorio_medicina_general.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Resumen" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Lista Unificada'!$A$4:$K$99</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Lista Unificada'!$A$4:$K$104</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -22,7 +22,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="$#,##0;($#,##0);-"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -71,6 +71,13 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00000000"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="000000FF"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -131,7 +138,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -170,8 +177,10 @@
     <xf numFmtId="164" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -257,6 +266,21 @@
     <comment ref="G5" authorId="0" shapeId="0">
       <text>
         <t>Precios aproximados de referencia (COP, 2026) a partir de rangos típicos de distribuidores de dispositivos médicos en Colombia, IVA incluido cuando aplica. Pueden variar ±20-30% según marca, proveedor y volumen. Validar con 2-3 cotizaciones formales.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Claude</author>
+  </authors>
+  <commentList>
+    <comment ref="B18" authorId="0" shapeId="0">
+      <text>
+        <t>Dato a confirmar: la lista del Dr. Durán indica que el consultorio 1104 necesita la misma dotación que el 1105-01. Ponga 2 si se cotizan ambos.</t>
       </text>
     </comment>
   </commentList>
@@ -552,7 +576,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K100"/>
+  <dimension ref="A1:K105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -578,7 +602,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Valores aproximados en pesos colombianos (COP), mercado colombiano 2026. Celdas amarillas = para diligenciar (ítems del Dr. Sergio Durán).</t>
+          <t>Valores aproximados en pesos colombianos (COP), mercado colombiano 2026. Incluye la lista del Dr. Sergio Durán (PDF “Dotación necesaria para los consultorios”). Celdas amarillas = ítems adicionales.</t>
         </is>
       </c>
     </row>
@@ -922,10 +946,14 @@
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>Dotación básica</t>
-        </is>
-      </c>
-      <c r="K10" s="5" t="inlineStr"/>
+          <t>Ambas</t>
+        </is>
+      </c>
+      <c r="K10" s="5" t="inlineStr">
+        <is>
+          <t>Dr. Durán: 'Termómetro' (botiquín)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
@@ -2786,10 +2814,14 @@
       </c>
       <c r="J50" s="4" t="inlineStr">
         <is>
-          <t>Dotación básica</t>
-        </is>
-      </c>
-      <c r="K50" s="5" t="inlineStr"/>
+          <t>Ambas</t>
+        </is>
+      </c>
+      <c r="K50" s="5" t="inlineStr">
+        <is>
+          <t>Dr. Durán pide el jabón y las toallas (ver Aseo)</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="n">
@@ -2878,10 +2910,14 @@
       </c>
       <c r="J52" s="4" t="inlineStr">
         <is>
-          <t>Dotación básica</t>
-        </is>
-      </c>
-      <c r="K52" s="5" t="inlineStr"/>
+          <t>Ambas</t>
+        </is>
+      </c>
+      <c r="K52" s="5" t="inlineStr">
+        <is>
+          <t>Dr. Durán: 'Guantes de examen' y 'Guantes desechables'</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="n">
@@ -3154,10 +3190,14 @@
       </c>
       <c r="J58" s="4" t="inlineStr">
         <is>
-          <t>Dotación básica</t>
-        </is>
-      </c>
-      <c r="K58" s="5" t="inlineStr"/>
+          <t>Ambas</t>
+        </is>
+      </c>
+      <c r="K58" s="5" t="inlineStr">
+        <is>
+          <t>Dr. Durán: gasas para retiro de puntos y botiquín</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="n">
@@ -3200,10 +3240,14 @@
       </c>
       <c r="J59" s="4" t="inlineStr">
         <is>
-          <t>Dotación básica</t>
-        </is>
-      </c>
-      <c r="K59" s="5" t="inlineStr"/>
+          <t>Ambas</t>
+        </is>
+      </c>
+      <c r="K59" s="5" t="inlineStr">
+        <is>
+          <t>Dr. Durán: botiquín</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="n">
@@ -3246,10 +3290,14 @@
       </c>
       <c r="J60" s="4" t="inlineStr">
         <is>
-          <t>Dotación básica</t>
-        </is>
-      </c>
-      <c r="K60" s="5" t="inlineStr"/>
+          <t>Ambas</t>
+        </is>
+      </c>
+      <c r="K60" s="5" t="inlineStr">
+        <is>
+          <t>Dr. Durán: botiquín</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="n">
@@ -3624,561 +3672,1185 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="9" t="inlineStr">
-        <is>
-          <t>Ítems enviados por el Dr. Sergio Durán (WhatsApp) — pendientes de transcribir</t>
+      <c r="A69" s="4" t="n">
+        <v>65</v>
+      </c>
+      <c r="B69" s="4" t="inlineStr">
+        <is>
+          <t>Atención de pacientes</t>
+        </is>
+      </c>
+      <c r="C69" s="5" t="inlineStr">
+        <is>
+          <t>Caja menor con llave</t>
+        </is>
+      </c>
+      <c r="D69" s="5" t="inlineStr">
+        <is>
+          <t>Metálica, para guardar dinero de caja chica</t>
+        </is>
+      </c>
+      <c r="E69" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F69" s="4" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="G69" s="7" t="n">
+        <v>80000</v>
+      </c>
+      <c r="H69" s="8">
+        <f>IF(OR(E69="",G69=""),"",E69*G69)</f>
+        <v/>
+      </c>
+      <c r="I69" s="4" t="inlineStr">
+        <is>
+          <t>Recomendado</t>
+        </is>
+      </c>
+      <c r="J69" s="4" t="inlineStr">
+        <is>
+          <t>Dr. Sergio Durán</t>
+        </is>
+      </c>
+      <c r="K69" s="5" t="inlineStr">
+        <is>
+          <t>Dr. Durán: 'Caja chica (para almacenamiento) – para guardar dinero'</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="4" t="n">
-        <v>65</v>
-      </c>
-      <c r="B70" s="10" t="inlineStr"/>
-      <c r="C70" s="11" t="inlineStr"/>
-      <c r="D70" s="11" t="inlineStr"/>
-      <c r="E70" s="10" t="n"/>
-      <c r="F70" s="10" t="inlineStr"/>
-      <c r="G70" s="12" t="n"/>
+        <v>66</v>
+      </c>
+      <c r="B70" s="4" t="inlineStr">
+        <is>
+          <t>Instrumental</t>
+        </is>
+      </c>
+      <c r="C70" s="5" t="inlineStr">
+        <is>
+          <t>Kit para retiro de puntos</t>
+        </is>
+      </c>
+      <c r="D70" s="5" t="inlineStr">
+        <is>
+          <t>Tijera de retiro de puntos (Spencer) + pinza de disección</t>
+        </is>
+      </c>
+      <c r="E70" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F70" s="4" t="inlineStr">
+        <is>
+          <t>Kit</t>
+        </is>
+      </c>
+      <c r="G70" s="7" t="n">
+        <v>60000</v>
+      </c>
       <c r="H70" s="8">
         <f>IF(OR(E70="",G70=""),"",E70*G70)</f>
         <v/>
       </c>
-      <c r="I70" s="10" t="inlineStr"/>
+      <c r="I70" s="4" t="inlineStr">
+        <is>
+          <t>Obligatorio</t>
+        </is>
+      </c>
       <c r="J70" s="4" t="inlineStr">
         <is>
           <t>Dr. Sergio Durán</t>
         </is>
       </c>
-      <c r="K70" s="11" t="inlineStr"/>
+      <c r="K70" s="5" t="inlineStr">
+        <is>
+          <t>Gasas incluidas en Consumibles; según protocolo</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="4" t="n">
-        <v>66</v>
-      </c>
-      <c r="B71" s="10" t="inlineStr"/>
-      <c r="C71" s="11" t="inlineStr"/>
-      <c r="D71" s="11" t="inlineStr"/>
-      <c r="E71" s="10" t="n"/>
-      <c r="F71" s="10" t="inlineStr"/>
-      <c r="G71" s="12" t="n"/>
+        <v>67</v>
+      </c>
+      <c r="B71" s="4" t="inlineStr">
+        <is>
+          <t>Papelería y oficina</t>
+        </is>
+      </c>
+      <c r="C71" s="5" t="inlineStr">
+        <is>
+          <t>Lapiceros, lápices y marcadores</t>
+        </is>
+      </c>
+      <c r="D71" s="5" t="inlineStr">
+        <is>
+          <t>Surtido (incluye resaltadores)</t>
+        </is>
+      </c>
+      <c r="E71" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F71" s="4" t="inlineStr">
+        <is>
+          <t>Lote</t>
+        </is>
+      </c>
+      <c r="G71" s="7" t="n">
+        <v>50000</v>
+      </c>
       <c r="H71" s="8">
         <f>IF(OR(E71="",G71=""),"",E71*G71)</f>
         <v/>
       </c>
-      <c r="I71" s="10" t="inlineStr"/>
+      <c r="I71" s="4" t="inlineStr">
+        <is>
+          <t>Obligatorio</t>
+        </is>
+      </c>
       <c r="J71" s="4" t="inlineStr">
         <is>
           <t>Dr. Sergio Durán</t>
         </is>
       </c>
-      <c r="K71" s="11" t="inlineStr"/>
+      <c r="K71" s="5" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="4" t="n">
-        <v>67</v>
-      </c>
-      <c r="B72" s="10" t="inlineStr"/>
-      <c r="C72" s="11" t="inlineStr"/>
-      <c r="D72" s="11" t="inlineStr"/>
-      <c r="E72" s="10" t="n"/>
-      <c r="F72" s="10" t="inlineStr"/>
-      <c r="G72" s="12" t="n"/>
+        <v>68</v>
+      </c>
+      <c r="B72" s="4" t="inlineStr">
+        <is>
+          <t>Papelería y oficina</t>
+        </is>
+      </c>
+      <c r="C72" s="5" t="inlineStr">
+        <is>
+          <t>Engrapadora (cosedora)</t>
+        </is>
+      </c>
+      <c r="D72" s="5" t="inlineStr">
+        <is>
+          <t>Con caja de ganchos</t>
+        </is>
+      </c>
+      <c r="E72" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F72" s="4" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="G72" s="7" t="n">
+        <v>25000</v>
+      </c>
       <c r="H72" s="8">
         <f>IF(OR(E72="",G72=""),"",E72*G72)</f>
         <v/>
       </c>
-      <c r="I72" s="10" t="inlineStr"/>
+      <c r="I72" s="4" t="inlineStr">
+        <is>
+          <t>Obligatorio</t>
+        </is>
+      </c>
       <c r="J72" s="4" t="inlineStr">
         <is>
           <t>Dr. Sergio Durán</t>
         </is>
       </c>
-      <c r="K72" s="11" t="inlineStr"/>
+      <c r="K72" s="5" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="4" t="n">
-        <v>68</v>
-      </c>
-      <c r="B73" s="10" t="inlineStr"/>
-      <c r="C73" s="11" t="inlineStr"/>
-      <c r="D73" s="11" t="inlineStr"/>
-      <c r="E73" s="10" t="n"/>
-      <c r="F73" s="10" t="inlineStr"/>
-      <c r="G73" s="12" t="n"/>
+        <v>69</v>
+      </c>
+      <c r="B73" s="4" t="inlineStr">
+        <is>
+          <t>Papelería y oficina</t>
+        </is>
+      </c>
+      <c r="C73" s="5" t="inlineStr">
+        <is>
+          <t>Clips para papel</t>
+        </is>
+      </c>
+      <c r="D73" s="5" t="inlineStr">
+        <is>
+          <t>Caja x100</t>
+        </is>
+      </c>
+      <c r="E73" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F73" s="4" t="inlineStr">
+        <is>
+          <t>Caja</t>
+        </is>
+      </c>
+      <c r="G73" s="7" t="n">
+        <v>5000</v>
+      </c>
       <c r="H73" s="8">
         <f>IF(OR(E73="",G73=""),"",E73*G73)</f>
         <v/>
       </c>
-      <c r="I73" s="10" t="inlineStr"/>
+      <c r="I73" s="4" t="inlineStr">
+        <is>
+          <t>Obligatorio</t>
+        </is>
+      </c>
       <c r="J73" s="4" t="inlineStr">
         <is>
           <t>Dr. Sergio Durán</t>
         </is>
       </c>
-      <c r="K73" s="11" t="inlineStr"/>
+      <c r="K73" s="5" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="4" t="n">
-        <v>69</v>
-      </c>
-      <c r="B74" s="10" t="inlineStr"/>
-      <c r="C74" s="11" t="inlineStr"/>
-      <c r="D74" s="11" t="inlineStr"/>
-      <c r="E74" s="10" t="n"/>
-      <c r="F74" s="10" t="inlineStr"/>
-      <c r="G74" s="12" t="n"/>
+        <v>70</v>
+      </c>
+      <c r="B74" s="4" t="inlineStr">
+        <is>
+          <t>Papelería y oficina</t>
+        </is>
+      </c>
+      <c r="C74" s="5" t="inlineStr">
+        <is>
+          <t>Sacaganchos</t>
+        </is>
+      </c>
+      <c r="D74" s="5" t="inlineStr">
+        <is>
+          <t>Metálico</t>
+        </is>
+      </c>
+      <c r="E74" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F74" s="4" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="G74" s="7" t="n">
+        <v>5000</v>
+      </c>
       <c r="H74" s="8">
         <f>IF(OR(E74="",G74=""),"",E74*G74)</f>
         <v/>
       </c>
-      <c r="I74" s="10" t="inlineStr"/>
+      <c r="I74" s="4" t="inlineStr">
+        <is>
+          <t>Obligatorio</t>
+        </is>
+      </c>
       <c r="J74" s="4" t="inlineStr">
         <is>
           <t>Dr. Sergio Durán</t>
         </is>
       </c>
-      <c r="K74" s="11" t="inlineStr"/>
+      <c r="K74" s="5" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="4" t="n">
-        <v>70</v>
-      </c>
-      <c r="B75" s="10" t="inlineStr"/>
-      <c r="C75" s="11" t="inlineStr"/>
-      <c r="D75" s="11" t="inlineStr"/>
-      <c r="E75" s="10" t="n"/>
-      <c r="F75" s="10" t="inlineStr"/>
-      <c r="G75" s="12" t="n"/>
+        <v>71</v>
+      </c>
+      <c r="B75" s="4" t="inlineStr">
+        <is>
+          <t>Papelería y oficina</t>
+        </is>
+      </c>
+      <c r="C75" s="5" t="inlineStr">
+        <is>
+          <t>Perforadora</t>
+        </is>
+      </c>
+      <c r="D75" s="5" t="inlineStr">
+        <is>
+          <t>2 huecos</t>
+        </is>
+      </c>
+      <c r="E75" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F75" s="4" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="G75" s="7" t="n">
+        <v>25000</v>
+      </c>
       <c r="H75" s="8">
         <f>IF(OR(E75="",G75=""),"",E75*G75)</f>
         <v/>
       </c>
-      <c r="I75" s="10" t="inlineStr"/>
+      <c r="I75" s="4" t="inlineStr">
+        <is>
+          <t>Obligatorio</t>
+        </is>
+      </c>
       <c r="J75" s="4" t="inlineStr">
         <is>
           <t>Dr. Sergio Durán</t>
         </is>
       </c>
-      <c r="K75" s="11" t="inlineStr"/>
+      <c r="K75" s="5" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="4" t="n">
-        <v>71</v>
-      </c>
-      <c r="B76" s="10" t="inlineStr"/>
-      <c r="C76" s="11" t="inlineStr"/>
-      <c r="D76" s="11" t="inlineStr"/>
-      <c r="E76" s="10" t="n"/>
-      <c r="F76" s="10" t="inlineStr"/>
-      <c r="G76" s="12" t="n"/>
+        <v>72</v>
+      </c>
+      <c r="B76" s="4" t="inlineStr">
+        <is>
+          <t>Papelería y oficina</t>
+        </is>
+      </c>
+      <c r="C76" s="5" t="inlineStr">
+        <is>
+          <t>Resma de papel tamaño carta</t>
+        </is>
+      </c>
+      <c r="D76" s="5" t="inlineStr">
+        <is>
+          <t>500 hojas, 75 g</t>
+        </is>
+      </c>
+      <c r="E76" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="F76" s="4" t="inlineStr">
+        <is>
+          <t>Resma</t>
+        </is>
+      </c>
+      <c r="G76" s="7" t="n">
+        <v>25000</v>
+      </c>
       <c r="H76" s="8">
         <f>IF(OR(E76="",G76=""),"",E76*G76)</f>
         <v/>
       </c>
-      <c r="I76" s="10" t="inlineStr"/>
+      <c r="I76" s="4" t="inlineStr">
+        <is>
+          <t>Obligatorio</t>
+        </is>
+      </c>
       <c r="J76" s="4" t="inlineStr">
         <is>
           <t>Dr. Sergio Durán</t>
         </is>
       </c>
-      <c r="K76" s="11" t="inlineStr"/>
+      <c r="K76" s="5" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="4" t="n">
-        <v>72</v>
-      </c>
-      <c r="B77" s="10" t="inlineStr"/>
-      <c r="C77" s="11" t="inlineStr"/>
-      <c r="D77" s="11" t="inlineStr"/>
-      <c r="E77" s="10" t="n"/>
-      <c r="F77" s="10" t="inlineStr"/>
-      <c r="G77" s="12" t="n"/>
+        <v>73</v>
+      </c>
+      <c r="B77" s="4" t="inlineStr">
+        <is>
+          <t>Papelería y oficina</t>
+        </is>
+      </c>
+      <c r="C77" s="5" t="inlineStr">
+        <is>
+          <t>Mostrador de sobres y carpetas</t>
+        </is>
+      </c>
+      <c r="D77" s="5" t="inlineStr">
+        <is>
+          <t>Organizador de escritorio / revistero</t>
+        </is>
+      </c>
+      <c r="E77" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F77" s="4" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="G77" s="7" t="n">
+        <v>60000</v>
+      </c>
       <c r="H77" s="8">
         <f>IF(OR(E77="",G77=""),"",E77*G77)</f>
         <v/>
       </c>
-      <c r="I77" s="10" t="inlineStr"/>
+      <c r="I77" s="4" t="inlineStr">
+        <is>
+          <t>Recomendado</t>
+        </is>
+      </c>
       <c r="J77" s="4" t="inlineStr">
         <is>
           <t>Dr. Sergio Durán</t>
         </is>
       </c>
-      <c r="K77" s="11" t="inlineStr"/>
+      <c r="K77" s="5" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="4" t="n">
-        <v>73</v>
-      </c>
-      <c r="B78" s="10" t="inlineStr"/>
-      <c r="C78" s="11" t="inlineStr"/>
-      <c r="D78" s="11" t="inlineStr"/>
-      <c r="E78" s="10" t="n"/>
-      <c r="F78" s="10" t="inlineStr"/>
-      <c r="G78" s="12" t="n"/>
+        <v>74</v>
+      </c>
+      <c r="B78" s="4" t="inlineStr">
+        <is>
+          <t>Papelería y oficina</t>
+        </is>
+      </c>
+      <c r="C78" s="5" t="inlineStr">
+        <is>
+          <t>Formatos de informes</t>
+        </is>
+      </c>
+      <c r="D78" s="5" t="inlineStr">
+        <is>
+          <t>Impresión de formatos (lote)</t>
+        </is>
+      </c>
+      <c r="E78" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F78" s="4" t="inlineStr">
+        <is>
+          <t>Lote</t>
+        </is>
+      </c>
+      <c r="G78" s="7" t="n">
+        <v>80000</v>
+      </c>
       <c r="H78" s="8">
         <f>IF(OR(E78="",G78=""),"",E78*G78)</f>
         <v/>
       </c>
-      <c r="I78" s="10" t="inlineStr"/>
+      <c r="I78" s="4" t="inlineStr">
+        <is>
+          <t>Obligatorio</t>
+        </is>
+      </c>
       <c r="J78" s="4" t="inlineStr">
         <is>
           <t>Dr. Sergio Durán</t>
         </is>
       </c>
-      <c r="K78" s="11" t="inlineStr"/>
+      <c r="K78" s="5" t="inlineStr">
+        <is>
+          <t>Depende de cantidad y tipo de formato</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="4" t="n">
-        <v>74</v>
-      </c>
-      <c r="B79" s="10" t="inlineStr"/>
-      <c r="C79" s="11" t="inlineStr"/>
-      <c r="D79" s="11" t="inlineStr"/>
-      <c r="E79" s="10" t="n"/>
-      <c r="F79" s="10" t="inlineStr"/>
-      <c r="G79" s="12" t="n"/>
+        <v>75</v>
+      </c>
+      <c r="B79" s="4" t="inlineStr">
+        <is>
+          <t>Papelería y oficina</t>
+        </is>
+      </c>
+      <c r="C79" s="5" t="inlineStr">
+        <is>
+          <t>Tinta para sello y almohadilla</t>
+        </is>
+      </c>
+      <c r="D79" s="5" t="inlineStr">
+        <is>
+          <t>Almohadilla + frasco de tinta</t>
+        </is>
+      </c>
+      <c r="E79" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F79" s="4" t="inlineStr">
+        <is>
+          <t>Juego</t>
+        </is>
+      </c>
+      <c r="G79" s="7" t="n">
+        <v>20000</v>
+      </c>
       <c r="H79" s="8">
         <f>IF(OR(E79="",G79=""),"",E79*G79)</f>
         <v/>
       </c>
-      <c r="I79" s="10" t="inlineStr"/>
+      <c r="I79" s="4" t="inlineStr">
+        <is>
+          <t>Recomendado</t>
+        </is>
+      </c>
       <c r="J79" s="4" t="inlineStr">
         <is>
           <t>Dr. Sergio Durán</t>
         </is>
       </c>
-      <c r="K79" s="11" t="inlineStr"/>
+      <c r="K79" s="5" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="4" t="n">
-        <v>75</v>
-      </c>
-      <c r="B80" s="10" t="inlineStr"/>
-      <c r="C80" s="11" t="inlineStr"/>
-      <c r="D80" s="11" t="inlineStr"/>
-      <c r="E80" s="10" t="n"/>
-      <c r="F80" s="10" t="inlineStr"/>
-      <c r="G80" s="12" t="n"/>
+        <v>76</v>
+      </c>
+      <c r="B80" s="4" t="inlineStr">
+        <is>
+          <t>Papelería y oficina</t>
+        </is>
+      </c>
+      <c r="C80" s="5" t="inlineStr">
+        <is>
+          <t>Tijeras de oficina</t>
+        </is>
+      </c>
+      <c r="D80" s="5" t="inlineStr">
+        <is>
+          <t>Punta roma</t>
+        </is>
+      </c>
+      <c r="E80" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F80" s="4" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="G80" s="7" t="n">
+        <v>8000</v>
+      </c>
       <c r="H80" s="8">
         <f>IF(OR(E80="",G80=""),"",E80*G80)</f>
         <v/>
       </c>
-      <c r="I80" s="10" t="inlineStr"/>
+      <c r="I80" s="4" t="inlineStr">
+        <is>
+          <t>Obligatorio</t>
+        </is>
+      </c>
       <c r="J80" s="4" t="inlineStr">
         <is>
           <t>Dr. Sergio Durán</t>
         </is>
       </c>
-      <c r="K80" s="11" t="inlineStr"/>
+      <c r="K80" s="5" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="4" t="n">
-        <v>76</v>
-      </c>
-      <c r="B81" s="10" t="inlineStr"/>
-      <c r="C81" s="11" t="inlineStr"/>
-      <c r="D81" s="11" t="inlineStr"/>
-      <c r="E81" s="10" t="n"/>
-      <c r="F81" s="10" t="inlineStr"/>
-      <c r="G81" s="12" t="n"/>
+        <v>77</v>
+      </c>
+      <c r="B81" s="4" t="inlineStr">
+        <is>
+          <t>Papelería y oficina</t>
+        </is>
+      </c>
+      <c r="C81" s="5" t="inlineStr">
+        <is>
+          <t>Cinta adhesiva</t>
+        </is>
+      </c>
+      <c r="D81" s="5" t="inlineStr">
+        <is>
+          <t>Rollo transparente</t>
+        </is>
+      </c>
+      <c r="E81" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="F81" s="4" t="inlineStr">
+        <is>
+          <t>Rollo</t>
+        </is>
+      </c>
+      <c r="G81" s="7" t="n">
+        <v>4000</v>
+      </c>
       <c r="H81" s="8">
         <f>IF(OR(E81="",G81=""),"",E81*G81)</f>
         <v/>
       </c>
-      <c r="I81" s="10" t="inlineStr"/>
+      <c r="I81" s="4" t="inlineStr">
+        <is>
+          <t>Obligatorio</t>
+        </is>
+      </c>
       <c r="J81" s="4" t="inlineStr">
         <is>
           <t>Dr. Sergio Durán</t>
         </is>
       </c>
-      <c r="K81" s="11" t="inlineStr"/>
+      <c r="K81" s="5" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="4" t="n">
-        <v>77</v>
-      </c>
-      <c r="B82" s="10" t="inlineStr"/>
-      <c r="C82" s="11" t="inlineStr"/>
-      <c r="D82" s="11" t="inlineStr"/>
-      <c r="E82" s="10" t="n"/>
-      <c r="F82" s="10" t="inlineStr"/>
-      <c r="G82" s="12" t="n"/>
+        <v>78</v>
+      </c>
+      <c r="B82" s="4" t="inlineStr">
+        <is>
+          <t>Papelería y oficina</t>
+        </is>
+      </c>
+      <c r="C82" s="5" t="inlineStr">
+        <is>
+          <t>Pegamento</t>
+        </is>
+      </c>
+      <c r="D82" s="5" t="inlineStr">
+        <is>
+          <t>Barra 40 g</t>
+        </is>
+      </c>
+      <c r="E82" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F82" s="4" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="G82" s="7" t="n">
+        <v>5000</v>
+      </c>
       <c r="H82" s="8">
         <f>IF(OR(E82="",G82=""),"",E82*G82)</f>
         <v/>
       </c>
-      <c r="I82" s="10" t="inlineStr"/>
+      <c r="I82" s="4" t="inlineStr">
+        <is>
+          <t>Obligatorio</t>
+        </is>
+      </c>
       <c r="J82" s="4" t="inlineStr">
         <is>
           <t>Dr. Sergio Durán</t>
         </is>
       </c>
-      <c r="K82" s="11" t="inlineStr"/>
+      <c r="K82" s="5" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="4" t="n">
-        <v>78</v>
-      </c>
-      <c r="B83" s="10" t="inlineStr"/>
-      <c r="C83" s="11" t="inlineStr"/>
-      <c r="D83" s="11" t="inlineStr"/>
-      <c r="E83" s="10" t="n"/>
-      <c r="F83" s="10" t="inlineStr"/>
-      <c r="G83" s="12" t="n"/>
+        <v>79</v>
+      </c>
+      <c r="B83" s="4" t="inlineStr">
+        <is>
+          <t>Papelería y oficina</t>
+        </is>
+      </c>
+      <c r="C83" s="5" t="inlineStr">
+        <is>
+          <t>Calculadora</t>
+        </is>
+      </c>
+      <c r="D83" s="5" t="inlineStr">
+        <is>
+          <t>De escritorio, 12 dígitos</t>
+        </is>
+      </c>
+      <c r="E83" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F83" s="4" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="G83" s="7" t="n">
+        <v>40000</v>
+      </c>
       <c r="H83" s="8">
         <f>IF(OR(E83="",G83=""),"",E83*G83)</f>
         <v/>
       </c>
-      <c r="I83" s="10" t="inlineStr"/>
+      <c r="I83" s="4" t="inlineStr">
+        <is>
+          <t>Recomendado</t>
+        </is>
+      </c>
       <c r="J83" s="4" t="inlineStr">
         <is>
           <t>Dr. Sergio Durán</t>
         </is>
       </c>
-      <c r="K83" s="11" t="inlineStr"/>
+      <c r="K83" s="5" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="4" t="n">
-        <v>79</v>
-      </c>
-      <c r="B84" s="10" t="inlineStr"/>
-      <c r="C84" s="11" t="inlineStr"/>
-      <c r="D84" s="11" t="inlineStr"/>
-      <c r="E84" s="10" t="n"/>
-      <c r="F84" s="10" t="inlineStr"/>
-      <c r="G84" s="12" t="n"/>
+        <v>80</v>
+      </c>
+      <c r="B84" s="4" t="inlineStr">
+        <is>
+          <t>Papelería y oficina</t>
+        </is>
+      </c>
+      <c r="C84" s="5" t="inlineStr">
+        <is>
+          <t>Libretas</t>
+        </is>
+      </c>
+      <c r="D84" s="5" t="inlineStr">
+        <is>
+          <t>Cuaderno / libreta de notas</t>
+        </is>
+      </c>
+      <c r="E84" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="F84" s="4" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="G84" s="7" t="n">
+        <v>6000</v>
+      </c>
       <c r="H84" s="8">
         <f>IF(OR(E84="",G84=""),"",E84*G84)</f>
         <v/>
       </c>
-      <c r="I84" s="10" t="inlineStr"/>
+      <c r="I84" s="4" t="inlineStr">
+        <is>
+          <t>Obligatorio</t>
+        </is>
+      </c>
       <c r="J84" s="4" t="inlineStr">
         <is>
           <t>Dr. Sergio Durán</t>
         </is>
       </c>
-      <c r="K84" s="11" t="inlineStr"/>
+      <c r="K84" s="5" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="4" t="n">
-        <v>80</v>
-      </c>
-      <c r="B85" s="10" t="inlineStr"/>
-      <c r="C85" s="11" t="inlineStr"/>
-      <c r="D85" s="11" t="inlineStr"/>
-      <c r="E85" s="10" t="n"/>
-      <c r="F85" s="10" t="inlineStr"/>
-      <c r="G85" s="12" t="n"/>
+        <v>81</v>
+      </c>
+      <c r="B85" s="4" t="inlineStr">
+        <is>
+          <t>Papelería y oficina</t>
+        </is>
+      </c>
+      <c r="C85" s="5" t="inlineStr">
+        <is>
+          <t>Repuestos (bolígrafos, etc.)</t>
+        </is>
+      </c>
+      <c r="D85" s="5" t="inlineStr">
+        <is>
+          <t>Minas, grapas, cartuchos varios</t>
+        </is>
+      </c>
+      <c r="E85" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F85" s="4" t="inlineStr">
+        <is>
+          <t>Lote</t>
+        </is>
+      </c>
+      <c r="G85" s="7" t="n">
+        <v>20000</v>
+      </c>
       <c r="H85" s="8">
         <f>IF(OR(E85="",G85=""),"",E85*G85)</f>
         <v/>
       </c>
-      <c r="I85" s="10" t="inlineStr"/>
+      <c r="I85" s="4" t="inlineStr">
+        <is>
+          <t>Recomendado</t>
+        </is>
+      </c>
       <c r="J85" s="4" t="inlineStr">
         <is>
           <t>Dr. Sergio Durán</t>
         </is>
       </c>
-      <c r="K85" s="11" t="inlineStr"/>
+      <c r="K85" s="5" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="4" t="n">
-        <v>81</v>
-      </c>
-      <c r="B86" s="10" t="inlineStr"/>
-      <c r="C86" s="11" t="inlineStr"/>
-      <c r="D86" s="11" t="inlineStr"/>
-      <c r="E86" s="10" t="n"/>
-      <c r="F86" s="10" t="inlineStr"/>
-      <c r="G86" s="12" t="n"/>
+        <v>82</v>
+      </c>
+      <c r="B86" s="4" t="inlineStr">
+        <is>
+          <t>Aseo y baño</t>
+        </is>
+      </c>
+      <c r="C86" s="5" t="inlineStr">
+        <is>
+          <t>Papel higiénico</t>
+        </is>
+      </c>
+      <c r="D86" s="5" t="inlineStr">
+        <is>
+          <t>Paquete x12 rollos institucional</t>
+        </is>
+      </c>
+      <c r="E86" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F86" s="4" t="inlineStr">
+        <is>
+          <t>Paquete</t>
+        </is>
+      </c>
+      <c r="G86" s="7" t="n">
+        <v>40000</v>
+      </c>
       <c r="H86" s="8">
         <f>IF(OR(E86="",G86=""),"",E86*G86)</f>
         <v/>
       </c>
-      <c r="I86" s="10" t="inlineStr"/>
+      <c r="I86" s="4" t="inlineStr">
+        <is>
+          <t>Obligatorio</t>
+        </is>
+      </c>
       <c r="J86" s="4" t="inlineStr">
         <is>
           <t>Dr. Sergio Durán</t>
         </is>
       </c>
-      <c r="K86" s="11" t="inlineStr"/>
+      <c r="K86" s="5" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="4" t="n">
-        <v>82</v>
-      </c>
-      <c r="B87" s="10" t="inlineStr"/>
-      <c r="C87" s="11" t="inlineStr"/>
-      <c r="D87" s="11" t="inlineStr"/>
-      <c r="E87" s="10" t="n"/>
-      <c r="F87" s="10" t="inlineStr"/>
-      <c r="G87" s="12" t="n"/>
+        <v>83</v>
+      </c>
+      <c r="B87" s="4" t="inlineStr">
+        <is>
+          <t>Aseo y baño</t>
+        </is>
+      </c>
+      <c r="C87" s="5" t="inlineStr">
+        <is>
+          <t>Jabón de manos</t>
+        </is>
+      </c>
+      <c r="D87" s="5" t="inlineStr">
+        <is>
+          <t>Líquido antibacterial, galón</t>
+        </is>
+      </c>
+      <c r="E87" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F87" s="4" t="inlineStr">
+        <is>
+          <t>Galón</t>
+        </is>
+      </c>
+      <c r="G87" s="7" t="n">
+        <v>35000</v>
+      </c>
       <c r="H87" s="8">
         <f>IF(OR(E87="",G87=""),"",E87*G87)</f>
         <v/>
       </c>
-      <c r="I87" s="10" t="inlineStr"/>
+      <c r="I87" s="4" t="inlineStr">
+        <is>
+          <t>Obligatorio</t>
+        </is>
+      </c>
       <c r="J87" s="4" t="inlineStr">
         <is>
           <t>Dr. Sergio Durán</t>
         </is>
       </c>
-      <c r="K87" s="11" t="inlineStr"/>
+      <c r="K87" s="5" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="4" t="n">
-        <v>83</v>
-      </c>
-      <c r="B88" s="10" t="inlineStr"/>
-      <c r="C88" s="11" t="inlineStr"/>
-      <c r="D88" s="11" t="inlineStr"/>
-      <c r="E88" s="10" t="n"/>
-      <c r="F88" s="10" t="inlineStr"/>
-      <c r="G88" s="12" t="n"/>
+        <v>84</v>
+      </c>
+      <c r="B88" s="4" t="inlineStr">
+        <is>
+          <t>Aseo y baño</t>
+        </is>
+      </c>
+      <c r="C88" s="5" t="inlineStr">
+        <is>
+          <t>Toallas de papel</t>
+        </is>
+      </c>
+      <c r="D88" s="5" t="inlineStr">
+        <is>
+          <t>Interfoliadas, paquete x150 (fardo)</t>
+        </is>
+      </c>
+      <c r="E88" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F88" s="4" t="inlineStr">
+        <is>
+          <t>Fardo</t>
+        </is>
+      </c>
+      <c r="G88" s="7" t="n">
+        <v>60000</v>
+      </c>
       <c r="H88" s="8">
         <f>IF(OR(E88="",G88=""),"",E88*G88)</f>
         <v/>
       </c>
-      <c r="I88" s="10" t="inlineStr"/>
+      <c r="I88" s="4" t="inlineStr">
+        <is>
+          <t>Obligatorio</t>
+        </is>
+      </c>
       <c r="J88" s="4" t="inlineStr">
         <is>
           <t>Dr. Sergio Durán</t>
         </is>
       </c>
-      <c r="K88" s="11" t="inlineStr"/>
+      <c r="K88" s="5" t="inlineStr">
+        <is>
+          <t>Se prefieren de papel sobre tela por bioseguridad</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="4" t="n">
-        <v>84</v>
-      </c>
-      <c r="B89" s="10" t="inlineStr"/>
-      <c r="C89" s="11" t="inlineStr"/>
-      <c r="D89" s="11" t="inlineStr"/>
-      <c r="E89" s="10" t="n"/>
-      <c r="F89" s="10" t="inlineStr"/>
-      <c r="G89" s="12" t="n"/>
+        <v>85</v>
+      </c>
+      <c r="B89" s="4" t="inlineStr">
+        <is>
+          <t>Aseo y baño</t>
+        </is>
+      </c>
+      <c r="C89" s="5" t="inlineStr">
+        <is>
+          <t>Ambientador</t>
+        </is>
+      </c>
+      <c r="D89" s="5" t="inlineStr">
+        <is>
+          <t>Aerosol</t>
+        </is>
+      </c>
+      <c r="E89" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F89" s="4" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="G89" s="7" t="n">
+        <v>15000</v>
+      </c>
       <c r="H89" s="8">
         <f>IF(OR(E89="",G89=""),"",E89*G89)</f>
         <v/>
       </c>
-      <c r="I89" s="10" t="inlineStr"/>
+      <c r="I89" s="4" t="inlineStr">
+        <is>
+          <t>Recomendado</t>
+        </is>
+      </c>
       <c r="J89" s="4" t="inlineStr">
         <is>
           <t>Dr. Sergio Durán</t>
         </is>
       </c>
-      <c r="K89" s="11" t="inlineStr"/>
+      <c r="K89" s="5" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="4" t="n">
-        <v>85</v>
-      </c>
-      <c r="B90" s="10" t="inlineStr"/>
-      <c r="C90" s="11" t="inlineStr"/>
-      <c r="D90" s="11" t="inlineStr"/>
-      <c r="E90" s="10" t="n"/>
-      <c r="F90" s="10" t="inlineStr"/>
-      <c r="G90" s="12" t="n"/>
+        <v>86</v>
+      </c>
+      <c r="B90" s="4" t="inlineStr">
+        <is>
+          <t>Botiquín de primeros auxilios</t>
+        </is>
+      </c>
+      <c r="C90" s="5" t="inlineStr">
+        <is>
+          <t>Botiquín</t>
+        </is>
+      </c>
+      <c r="D90" s="5" t="inlineStr">
+        <is>
+          <t>Gabinete o maletín con compartimentos</t>
+        </is>
+      </c>
+      <c r="E90" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F90" s="4" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="G90" s="7" t="n">
+        <v>60000</v>
+      </c>
       <c r="H90" s="8">
         <f>IF(OR(E90="",G90=""),"",E90*G90)</f>
         <v/>
       </c>
-      <c r="I90" s="10" t="inlineStr"/>
+      <c r="I90" s="4" t="inlineStr">
+        <is>
+          <t>Obligatorio</t>
+        </is>
+      </c>
       <c r="J90" s="4" t="inlineStr">
         <is>
           <t>Dr. Sergio Durán</t>
         </is>
       </c>
-      <c r="K90" s="11" t="inlineStr"/>
+      <c r="K90" s="5" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="4" t="n">
-        <v>86</v>
-      </c>
-      <c r="B91" s="10" t="inlineStr"/>
-      <c r="C91" s="11" t="inlineStr"/>
-      <c r="D91" s="11" t="inlineStr"/>
-      <c r="E91" s="10" t="n"/>
-      <c r="F91" s="10" t="inlineStr"/>
-      <c r="G91" s="12" t="n"/>
+        <v>87</v>
+      </c>
+      <c r="B91" s="4" t="inlineStr">
+        <is>
+          <t>Botiquín de primeros auxilios</t>
+        </is>
+      </c>
+      <c r="C91" s="5" t="inlineStr">
+        <is>
+          <t>Curitas</t>
+        </is>
+      </c>
+      <c r="D91" s="5" t="inlineStr">
+        <is>
+          <t>Caja x100</t>
+        </is>
+      </c>
+      <c r="E91" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F91" s="4" t="inlineStr">
+        <is>
+          <t>Caja</t>
+        </is>
+      </c>
+      <c r="G91" s="7" t="n">
+        <v>15000</v>
+      </c>
       <c r="H91" s="8">
         <f>IF(OR(E91="",G91=""),"",E91*G91)</f>
         <v/>
       </c>
-      <c r="I91" s="10" t="inlineStr"/>
+      <c r="I91" s="4" t="inlineStr">
+        <is>
+          <t>Obligatorio</t>
+        </is>
+      </c>
       <c r="J91" s="4" t="inlineStr">
         <is>
           <t>Dr. Sergio Durán</t>
         </is>
       </c>
-      <c r="K91" s="11" t="inlineStr"/>
+      <c r="K91" s="5" t="inlineStr">
+        <is>
+          <t>Gasas, algodón, guantes, termómetro y alcohol ya están en la lista</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="4" t="n">
-        <v>87</v>
-      </c>
-      <c r="B92" s="10" t="inlineStr"/>
-      <c r="C92" s="11" t="inlineStr"/>
-      <c r="D92" s="11" t="inlineStr"/>
-      <c r="E92" s="10" t="n"/>
-      <c r="F92" s="10" t="inlineStr"/>
-      <c r="G92" s="12" t="n"/>
+        <v>88</v>
+      </c>
+      <c r="B92" s="4" t="inlineStr">
+        <is>
+          <t>Botiquín de primeros auxilios</t>
+        </is>
+      </c>
+      <c r="C92" s="5" t="inlineStr">
+        <is>
+          <t>Medicamentos básicos</t>
+        </is>
+      </c>
+      <c r="D92" s="5" t="inlineStr">
+        <is>
+          <t>Acetaminofén, loratadina, sales de rehidratación, antiácido</t>
+        </is>
+      </c>
+      <c r="E92" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F92" s="4" t="inlineStr">
+        <is>
+          <t>Lote</t>
+        </is>
+      </c>
+      <c r="G92" s="7" t="n">
+        <v>100000</v>
+      </c>
       <c r="H92" s="8">
         <f>IF(OR(E92="",G92=""),"",E92*G92)</f>
         <v/>
       </c>
-      <c r="I92" s="10" t="inlineStr"/>
+      <c r="I92" s="4" t="inlineStr">
+        <is>
+          <t>Recomendado</t>
+        </is>
+      </c>
       <c r="J92" s="4" t="inlineStr">
         <is>
           <t>Dr. Sergio Durán</t>
         </is>
       </c>
-      <c r="K92" s="11" t="inlineStr"/>
+      <c r="K92" s="5" t="inlineStr">
+        <is>
+          <t>Definir listado con el Dr. Durán</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="4" t="n">
-        <v>88</v>
-      </c>
-      <c r="B93" s="10" t="inlineStr"/>
-      <c r="C93" s="11" t="inlineStr"/>
-      <c r="D93" s="11" t="inlineStr"/>
-      <c r="E93" s="10" t="n"/>
-      <c r="F93" s="10" t="inlineStr"/>
-      <c r="G93" s="12" t="n"/>
+        <v>89</v>
+      </c>
+      <c r="B93" s="4" t="inlineStr">
+        <is>
+          <t>Botiquín de primeros auxilios</t>
+        </is>
+      </c>
+      <c r="C93" s="5" t="inlineStr">
+        <is>
+          <t>Ibuprofeno 400 mg</t>
+        </is>
+      </c>
+      <c r="D93" s="5" t="inlineStr">
+        <is>
+          <t>Caja x50 tabletas</t>
+        </is>
+      </c>
+      <c r="E93" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F93" s="4" t="inlineStr">
+        <is>
+          <t>Caja</t>
+        </is>
+      </c>
+      <c r="G93" s="7" t="n">
+        <v>15000</v>
+      </c>
       <c r="H93" s="8">
         <f>IF(OR(E93="",G93=""),"",E93*G93)</f>
         <v/>
       </c>
-      <c r="I93" s="10" t="inlineStr"/>
+      <c r="I93" s="4" t="inlineStr">
+        <is>
+          <t>Recomendado</t>
+        </is>
+      </c>
       <c r="J93" s="4" t="inlineStr">
         <is>
           <t>Dr. Sergio Durán</t>
         </is>
       </c>
-      <c r="K93" s="11" t="inlineStr"/>
+      <c r="K93" s="5" t="inlineStr"/>
     </row>
     <row r="94">
-      <c r="A94" s="4" t="n">
-        <v>89</v>
-      </c>
-      <c r="B94" s="10" t="inlineStr"/>
-      <c r="C94" s="11" t="inlineStr"/>
-      <c r="D94" s="11" t="inlineStr"/>
-      <c r="E94" s="10" t="n"/>
-      <c r="F94" s="10" t="inlineStr"/>
-      <c r="G94" s="12" t="n"/>
-      <c r="H94" s="8">
-        <f>IF(OR(E94="",G94=""),"",E94*G94)</f>
-        <v/>
-      </c>
-      <c r="I94" s="10" t="inlineStr"/>
-      <c r="J94" s="4" t="inlineStr">
-        <is>
-          <t>Dr. Sergio Durán</t>
-        </is>
-      </c>
-      <c r="K94" s="11" t="inlineStr"/>
+      <c r="A94" s="9" t="inlineStr">
+        <is>
+          <t>Filas libres para ítems adicionales</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="4" t="n">
@@ -4195,11 +4867,7 @@
         <v/>
       </c>
       <c r="I95" s="10" t="inlineStr"/>
-      <c r="J95" s="4" t="inlineStr">
-        <is>
-          <t>Dr. Sergio Durán</t>
-        </is>
-      </c>
+      <c r="J95" s="4" t="inlineStr"/>
       <c r="K95" s="11" t="inlineStr"/>
     </row>
     <row r="96">
@@ -4217,11 +4885,7 @@
         <v/>
       </c>
       <c r="I96" s="10" t="inlineStr"/>
-      <c r="J96" s="4" t="inlineStr">
-        <is>
-          <t>Dr. Sergio Durán</t>
-        </is>
-      </c>
+      <c r="J96" s="4" t="inlineStr"/>
       <c r="K96" s="11" t="inlineStr"/>
     </row>
     <row r="97">
@@ -4239,11 +4903,7 @@
         <v/>
       </c>
       <c r="I97" s="10" t="inlineStr"/>
-      <c r="J97" s="4" t="inlineStr">
-        <is>
-          <t>Dr. Sergio Durán</t>
-        </is>
-      </c>
+      <c r="J97" s="4" t="inlineStr"/>
       <c r="K97" s="11" t="inlineStr"/>
     </row>
     <row r="98">
@@ -4261,11 +4921,7 @@
         <v/>
       </c>
       <c r="I98" s="10" t="inlineStr"/>
-      <c r="J98" s="4" t="inlineStr">
-        <is>
-          <t>Dr. Sergio Durán</t>
-        </is>
-      </c>
+      <c r="J98" s="4" t="inlineStr"/>
       <c r="K98" s="11" t="inlineStr"/>
     </row>
     <row r="99">
@@ -4283,31 +4939,117 @@
         <v/>
       </c>
       <c r="I99" s="10" t="inlineStr"/>
-      <c r="J99" s="4" t="inlineStr">
-        <is>
-          <t>Dr. Sergio Durán</t>
-        </is>
-      </c>
+      <c r="J99" s="4" t="inlineStr"/>
       <c r="K99" s="11" t="inlineStr"/>
     </row>
     <row r="100">
-      <c r="G100" s="13" t="inlineStr">
+      <c r="A100" s="4" t="n">
+        <v>95</v>
+      </c>
+      <c r="B100" s="10" t="inlineStr"/>
+      <c r="C100" s="11" t="inlineStr"/>
+      <c r="D100" s="11" t="inlineStr"/>
+      <c r="E100" s="10" t="n"/>
+      <c r="F100" s="10" t="inlineStr"/>
+      <c r="G100" s="12" t="n"/>
+      <c r="H100" s="8">
+        <f>IF(OR(E100="",G100=""),"",E100*G100)</f>
+        <v/>
+      </c>
+      <c r="I100" s="10" t="inlineStr"/>
+      <c r="J100" s="4" t="inlineStr"/>
+      <c r="K100" s="11" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="4" t="n">
+        <v>96</v>
+      </c>
+      <c r="B101" s="10" t="inlineStr"/>
+      <c r="C101" s="11" t="inlineStr"/>
+      <c r="D101" s="11" t="inlineStr"/>
+      <c r="E101" s="10" t="n"/>
+      <c r="F101" s="10" t="inlineStr"/>
+      <c r="G101" s="12" t="n"/>
+      <c r="H101" s="8">
+        <f>IF(OR(E101="",G101=""),"",E101*G101)</f>
+        <v/>
+      </c>
+      <c r="I101" s="10" t="inlineStr"/>
+      <c r="J101" s="4" t="inlineStr"/>
+      <c r="K101" s="11" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="4" t="n">
+        <v>97</v>
+      </c>
+      <c r="B102" s="10" t="inlineStr"/>
+      <c r="C102" s="11" t="inlineStr"/>
+      <c r="D102" s="11" t="inlineStr"/>
+      <c r="E102" s="10" t="n"/>
+      <c r="F102" s="10" t="inlineStr"/>
+      <c r="G102" s="12" t="n"/>
+      <c r="H102" s="8">
+        <f>IF(OR(E102="",G102=""),"",E102*G102)</f>
+        <v/>
+      </c>
+      <c r="I102" s="10" t="inlineStr"/>
+      <c r="J102" s="4" t="inlineStr"/>
+      <c r="K102" s="11" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="4" t="n">
+        <v>98</v>
+      </c>
+      <c r="B103" s="10" t="inlineStr"/>
+      <c r="C103" s="11" t="inlineStr"/>
+      <c r="D103" s="11" t="inlineStr"/>
+      <c r="E103" s="10" t="n"/>
+      <c r="F103" s="10" t="inlineStr"/>
+      <c r="G103" s="12" t="n"/>
+      <c r="H103" s="8">
+        <f>IF(OR(E103="",G103=""),"",E103*G103)</f>
+        <v/>
+      </c>
+      <c r="I103" s="10" t="inlineStr"/>
+      <c r="J103" s="4" t="inlineStr"/>
+      <c r="K103" s="11" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="4" t="n">
+        <v>99</v>
+      </c>
+      <c r="B104" s="10" t="inlineStr"/>
+      <c r="C104" s="11" t="inlineStr"/>
+      <c r="D104" s="11" t="inlineStr"/>
+      <c r="E104" s="10" t="n"/>
+      <c r="F104" s="10" t="inlineStr"/>
+      <c r="G104" s="12" t="n"/>
+      <c r="H104" s="8">
+        <f>IF(OR(E104="",G104=""),"",E104*G104)</f>
+        <v/>
+      </c>
+      <c r="I104" s="10" t="inlineStr"/>
+      <c r="J104" s="4" t="inlineStr"/>
+      <c r="K104" s="11" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="G105" s="13" t="inlineStr">
         <is>
           <t>TOTAL APROX.</t>
         </is>
       </c>
-      <c r="H100" s="14">
-        <f>SUM(H5:H99)</f>
+      <c r="H105" s="14">
+        <f>SUM(H5:H104)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:K99"/>
+  <autoFilter ref="A4:K104"/>
   <mergeCells count="1">
-    <mergeCell ref="A69:K69"/>
+    <mergeCell ref="A94:K94"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="I5:I99" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I5:I104" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Obligatorio,Recomendado,Opcional"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4322,7 +5064,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B29"/>
+  <dimension ref="A1:B38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -4355,7 +5097,7 @@
         </is>
       </c>
       <c r="B4" s="17">
-        <f>SUMIFS('Lista Unificada'!$H$5:$H$99,'Lista Unificada'!$B$5:$B$99,A4)</f>
+        <f>SUMIFS('Lista Unificada'!$H$5:$H$104,'Lista Unificada'!$B$5:$B$104,A4)</f>
         <v/>
       </c>
     </row>
@@ -4366,7 +5108,7 @@
         </is>
       </c>
       <c r="B5" s="17">
-        <f>SUMIFS('Lista Unificada'!$H$5:$H$99,'Lista Unificada'!$B$5:$B$99,A5)</f>
+        <f>SUMIFS('Lista Unificada'!$H$5:$H$104,'Lista Unificada'!$B$5:$B$104,A5)</f>
         <v/>
       </c>
     </row>
@@ -4377,7 +5119,7 @@
         </is>
       </c>
       <c r="B6" s="17">
-        <f>SUMIFS('Lista Unificada'!$H$5:$H$99,'Lista Unificada'!$B$5:$B$99,A6)</f>
+        <f>SUMIFS('Lista Unificada'!$H$5:$H$104,'Lista Unificada'!$B$5:$B$104,A6)</f>
         <v/>
       </c>
     </row>
@@ -4388,7 +5130,7 @@
         </is>
       </c>
       <c r="B7" s="17">
-        <f>SUMIFS('Lista Unificada'!$H$5:$H$99,'Lista Unificada'!$B$5:$B$99,A7)</f>
+        <f>SUMIFS('Lista Unificada'!$H$5:$H$104,'Lista Unificada'!$B$5:$B$104,A7)</f>
         <v/>
       </c>
     </row>
@@ -4399,7 +5141,7 @@
         </is>
       </c>
       <c r="B8" s="17">
-        <f>SUMIFS('Lista Unificada'!$H$5:$H$99,'Lista Unificada'!$B$5:$B$99,A8)</f>
+        <f>SUMIFS('Lista Unificada'!$H$5:$H$104,'Lista Unificada'!$B$5:$B$104,A8)</f>
         <v/>
       </c>
     </row>
@@ -4410,7 +5152,7 @@
         </is>
       </c>
       <c r="B9" s="17">
-        <f>SUMIFS('Lista Unificada'!$H$5:$H$99,'Lista Unificada'!$B$5:$B$99,A9)</f>
+        <f>SUMIFS('Lista Unificada'!$H$5:$H$104,'Lista Unificada'!$B$5:$B$104,A9)</f>
         <v/>
       </c>
     </row>
@@ -4421,7 +5163,7 @@
         </is>
       </c>
       <c r="B10" s="17">
-        <f>SUMIFS('Lista Unificada'!$H$5:$H$99,'Lista Unificada'!$B$5:$B$99,A10)</f>
+        <f>SUMIFS('Lista Unificada'!$H$5:$H$104,'Lista Unificada'!$B$5:$B$104,A10)</f>
         <v/>
       </c>
     </row>
@@ -4432,154 +5174,245 @@
         </is>
       </c>
       <c r="B11" s="17">
-        <f>SUMIFS('Lista Unificada'!$H$5:$H$99,'Lista Unificada'!$B$5:$B$99,A11)</f>
+        <f>SUMIFS('Lista Unificada'!$H$5:$H$104,'Lista Unificada'!$B$5:$B$104,A11)</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="16" t="inlineStr">
         <is>
-          <t>Otras categorías / sin clasificar</t>
+          <t>Atención de pacientes</t>
         </is>
       </c>
       <c r="B12" s="17">
-        <f>'Lista Unificada'!H100-SUM(B4:B11)</f>
+        <f>SUMIFS('Lista Unificada'!$H$5:$H$104,'Lista Unificada'!$B$5:$B$104,A12)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="18" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B13" s="19">
-        <f>'Lista Unificada'!H100</f>
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t>Papelería y oficina</t>
+        </is>
+      </c>
+      <c r="B13" s="17">
+        <f>SUMIFS('Lista Unificada'!$H$5:$H$104,'Lista Unificada'!$B$5:$B$104,A13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>Aseo y baño</t>
+        </is>
+      </c>
+      <c r="B14" s="17">
+        <f>SUMIFS('Lista Unificada'!$H$5:$H$104,'Lista Unificada'!$B$5:$B$104,A14)</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="15" t="inlineStr">
-        <is>
-          <t>Por fuente</t>
-        </is>
-      </c>
-      <c r="B15" s="15" t="inlineStr">
-        <is>
-          <t>Valor aprox. (COP)</t>
-        </is>
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t>Botiquín de primeros auxilios</t>
+        </is>
+      </c>
+      <c r="B15" s="17">
+        <f>SUMIFS('Lista Unificada'!$H$5:$H$104,'Lista Unificada'!$B$5:$B$104,A15)</f>
+        <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="16" t="inlineStr">
         <is>
-          <t>Dotación básica</t>
+          <t>Otras categorías / sin clasificar</t>
         </is>
       </c>
       <c r="B16" s="17">
-        <f>SUMIFS('Lista Unificada'!$H$5:$H$99,'Lista Unificada'!$J$5:$J$99,A16)</f>
+        <f>'Lista Unificada'!H105-SUM(B4:B15)</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="16" t="inlineStr">
-        <is>
-          <t>Dr. Sergio Durán</t>
-        </is>
-      </c>
-      <c r="B17" s="17">
-        <f>SUMIFS('Lista Unificada'!$H$5:$H$99,'Lista Unificada'!$J$5:$J$99,A17)</f>
-        <v/>
+      <c r="A17" s="18" t="inlineStr">
+        <is>
+          <t>TOTAL (1 consultorio)</t>
+        </is>
+      </c>
+      <c r="B17" s="19">
+        <f>'Lista Unificada'!H105</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="20" t="inlineStr">
+        <is>
+          <t>Consultorios a dotar</t>
+        </is>
+      </c>
+      <c r="B18" s="21" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="15" t="inlineStr">
-        <is>
-          <t>Por prioridad</t>
-        </is>
-      </c>
-      <c r="B19" s="15" t="inlineStr">
+      <c r="A19" s="18" t="inlineStr">
+        <is>
+          <t>TOTAL GENERAL</t>
+        </is>
+      </c>
+      <c r="B19" s="19">
+        <f>B17*B18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>Por fuente</t>
+        </is>
+      </c>
+      <c r="B21" s="15" t="inlineStr">
         <is>
           <t>Valor aprox. (COP)</t>
         </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="16" t="inlineStr">
-        <is>
-          <t>Obligatorio</t>
-        </is>
-      </c>
-      <c r="B20" s="17">
-        <f>SUMIFS('Lista Unificada'!$H$5:$H$99,'Lista Unificada'!$I$5:$I$99,A20)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="16" t="inlineStr">
-        <is>
-          <t>Recomendado</t>
-        </is>
-      </c>
-      <c r="B21" s="17">
-        <f>SUMIFS('Lista Unificada'!$H$5:$H$99,'Lista Unificada'!$I$5:$I$99,A21)</f>
-        <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="16" t="inlineStr">
         <is>
+          <t>Dotación básica</t>
+        </is>
+      </c>
+      <c r="B22" s="17">
+        <f>SUMIFS('Lista Unificada'!$H$5:$H$104,'Lista Unificada'!$J$5:$J$104,A22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="16" t="inlineStr">
+        <is>
+          <t>Dr. Sergio Durán</t>
+        </is>
+      </c>
+      <c r="B23" s="17">
+        <f>SUMIFS('Lista Unificada'!$H$5:$H$104,'Lista Unificada'!$J$5:$J$104,A23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="16" t="inlineStr">
+        <is>
+          <t>Ambas</t>
+        </is>
+      </c>
+      <c r="B24" s="17">
+        <f>SUMIFS('Lista Unificada'!$H$5:$H$104,'Lista Unificada'!$J$5:$J$104,A24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="15" t="inlineStr">
+        <is>
+          <t>Por prioridad</t>
+        </is>
+      </c>
+      <c r="B26" s="15" t="inlineStr">
+        <is>
+          <t>Valor aprox. (COP)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="16" t="inlineStr">
+        <is>
+          <t>Obligatorio</t>
+        </is>
+      </c>
+      <c r="B27" s="17">
+        <f>SUMIFS('Lista Unificada'!$H$5:$H$104,'Lista Unificada'!$I$5:$I$104,A27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="16" t="inlineStr">
+        <is>
+          <t>Recomendado</t>
+        </is>
+      </c>
+      <c r="B28" s="17">
+        <f>SUMIFS('Lista Unificada'!$H$5:$H$104,'Lista Unificada'!$I$5:$I$104,A28)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="16" t="inlineStr">
+        <is>
           <t>Opcional</t>
         </is>
       </c>
-      <c r="B22" s="17">
-        <f>SUMIFS('Lista Unificada'!$H$5:$H$99,'Lista Unificada'!$I$5:$I$99,A22)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="20" t="inlineStr">
+      <c r="B29" s="17">
+        <f>SUMIFS('Lista Unificada'!$H$5:$H$104,'Lista Unificada'!$I$5:$I$104,A29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="22" t="inlineStr">
         <is>
           <t>Notas y supuestos:</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="21" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="23" t="inlineStr">
         <is>
           <t>• Valores aproximados en COP (2026), referencia de distribuidores de dispositivos médicos en Colombia; variación esperada ±20-30%.</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="21" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="23" t="inlineStr">
         <is>
           <t>• Prioridad orientativa según requisitos típicos de habilitación de consulta externa de medicina general (Resolución 3100 de 2019); verificar con la Secretaría de Salud.</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="21" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="23" t="inlineStr">
         <is>
           <t>• Los equipos biomédicos requieren registro INVIMA, hoja de vida y plan de mantenimiento/calibración.</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="21" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="23" t="inlineStr">
         <is>
           <t>• Cantidades pensadas para 1 consultorio y dotación inicial de consumibles (~1 mes).</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="21" t="inlineStr">
-        <is>
-          <t>• Para diligenciar: filas amarillas de 'Lista Unificada' (ítems del Dr. Sergio Durán). El total se actualiza solo.</t>
+    <row r="36">
+      <c r="A36" s="23" t="inlineStr">
+        <is>
+          <t>• Fuente 'Ambas' = ítem pedido por el Dr. Durán que ya estaba en la dotación básica (se unificó sin duplicar).</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="23" t="inlineStr">
+        <is>
+          <t>• Según el Dr. Durán, el consultorio 1104 necesita la misma dotación que el 1105-01. Ajuste 'Consultorios a dotar' arriba.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="23" t="inlineStr">
+        <is>
+          <t>• Filas amarillas de 'Lista Unificada' = ítems adicionales; el total se actualiza solo.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>